<commit_message>
chore: push pending UI, packaging, and rate fixes
</commit_message>
<xml_diff>
--- a/WORKINGS FOR CURT APP PRICING.xlsx 20-05-2026.xlsx
+++ b/WORKINGS FOR CURT APP PRICING.xlsx 20-05-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Accounts\OneDrive\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curt/Desktop/CSA /Clients/Master Movers /Master Movers APP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879394DB-30B8-4CF9-B2E7-35B7C92B2784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3AA3CF-2C82-DA4C-85C2-191D00D531EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1068" windowWidth="23040" windowHeight="11892" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-10020" windowWidth="38400" windowHeight="21600" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="National Costing" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="125">
   <si>
     <t>Route</t>
   </si>
@@ -381,9 +381,6 @@
     <t>Minimum</t>
   </si>
   <si>
-    <t>Flat rate of  30 - 50 M @R450</t>
-  </si>
-  <si>
     <t>Flat Rate    50M and over needs shuttle</t>
   </si>
   <si>
@@ -400,6 +397,21 @@
   </si>
   <si>
     <t>R2 600.00</t>
+  </si>
+  <si>
+    <t>Flat rate of  50-80 M @R450</t>
+  </si>
+  <si>
+    <t>Long Carry Stairs</t>
+  </si>
+  <si>
+    <t>2nd floor R450, Above 3-4th floor R750, higher than 5th R950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoisting </t>
+  </si>
+  <si>
+    <t xml:space="preserve">R850 flat rate </t>
   </si>
 </sst>
 </file>
@@ -407,9 +419,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0_);[Red]\(&quot;R&quot;#,##0\)"/>
-    <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="#.##0.00"/>
+    <numFmt numFmtId="6" formatCode="&quot;R&quot;#,##0_);[Red]\(&quot;R&quot;#,##0\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#.##0.00"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -684,12 +696,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -707,8 +719,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -729,7 +741,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
@@ -738,7 +750,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -756,7 +768,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -792,6 +804,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,24 +1112,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M69"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
     <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="8" max="8" width="14.5" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="7.6640625" customWidth="1"/>
     <col min="11" max="11" width="76" customWidth="1"/>
-    <col min="12" max="12" width="14.44140625" customWidth="1"/>
-    <col min="13" max="13" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5" customWidth="1"/>
+    <col min="13" max="13" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
         <v>40</v>
       </c>
@@ -1128,7 +1145,7 @@
       <c r="J1" s="49"/>
       <c r="K1" s="49"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1163,7 +1180,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -1176,7 +1193,7 @@
       <c r="K3" s="31"/>
       <c r="L3" s="34"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
@@ -1207,7 +1224,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
@@ -1239,7 +1256,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
@@ -1267,7 +1284,7 @@
       </c>
       <c r="L6" s="35"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
@@ -1291,11 +1308,11 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L7" s="35"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
@@ -1319,7 +1336,7 @@
       <c r="K8" s="14"/>
       <c r="L8" s="35"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
@@ -1343,7 +1360,7 @@
       <c r="K9" s="14"/>
       <c r="L9" s="35"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
@@ -1367,7 +1384,7 @@
       <c r="K10" s="14"/>
       <c r="L10" s="35"/>
     </row>
-    <row r="11" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -1393,7 +1410,7 @@
       </c>
       <c r="L11" s="35"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
@@ -1417,7 +1434,7 @@
       <c r="K12" s="14"/>
       <c r="L12" s="35"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -1430,7 +1447,7 @@
       <c r="K13" s="14"/>
       <c r="L13" s="35"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -1443,7 +1460,7 @@
       <c r="K14" s="14"/>
       <c r="L14" s="35"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="13"/>
@@ -1455,7 +1472,7 @@
       <c r="K15" s="15"/>
       <c r="L15" s="36"/>
     </row>
-    <row r="18" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="53" t="s">
         <v>41</v>
       </c>
@@ -1473,7 +1490,7 @@
       <c r="L18" s="55"/>
       <c r="M18" s="56"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
@@ -1511,7 +1528,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1525,7 +1542,7 @@
       <c r="L20" s="21"/>
       <c r="M20" s="21"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>42</v>
       </c>
@@ -1559,7 +1576,7 @@
       </c>
       <c r="M21" s="25"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>43</v>
       </c>
@@ -1593,7 +1610,7 @@
       </c>
       <c r="M22" s="25"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>44</v>
       </c>
@@ -1627,7 +1644,7 @@
       </c>
       <c r="M23" s="25"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>45</v>
       </c>
@@ -1661,7 +1678,7 @@
       </c>
       <c r="M24" s="25"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>46</v>
       </c>
@@ -1687,7 +1704,7 @@
       <c r="L25" s="25"/>
       <c r="M25" s="25"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>47</v>
       </c>
@@ -1713,7 +1730,7 @@
       <c r="L26" s="25"/>
       <c r="M26" s="25"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>48</v>
       </c>
@@ -1739,7 +1756,7 @@
       <c r="L27" s="25"/>
       <c r="M27" s="25"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>49</v>
       </c>
@@ -1765,7 +1782,7 @@
       <c r="L28" s="25"/>
       <c r="M28" s="25"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>50</v>
       </c>
@@ -1791,7 +1808,7 @@
       <c r="L29" s="25"/>
       <c r="M29" s="25"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>97</v>
       </c>
@@ -1815,10 +1832,10 @@
       <c r="L30" s="28"/>
       <c r="M30" s="28"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="7"/>
     </row>
-    <row r="34" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" ht="19" x14ac:dyDescent="0.25">
       <c r="A34" s="53" t="s">
         <v>51</v>
       </c>
@@ -1836,7 +1853,7 @@
       <c r="L34" s="55"/>
       <c r="M34" s="56"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>0</v>
       </c>
@@ -1874,7 +1891,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -1888,7 +1905,7 @@
       <c r="L36" s="46"/>
       <c r="M36" s="21"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>42</v>
       </c>
@@ -1922,7 +1939,7 @@
       </c>
       <c r="M37" s="25"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>43</v>
       </c>
@@ -1956,7 +1973,7 @@
       </c>
       <c r="M38" s="25"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>44</v>
       </c>
@@ -1990,7 +2007,7 @@
       </c>
       <c r="M39" s="25"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>45</v>
       </c>
@@ -2024,7 +2041,7 @@
       </c>
       <c r="M40" s="25"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
         <v>46</v>
       </c>
@@ -2058,7 +2075,7 @@
       </c>
       <c r="M41" s="25"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
         <v>47</v>
       </c>
@@ -2082,7 +2099,7 @@
       <c r="L42" s="44"/>
       <c r="M42" s="25"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
@@ -2096,7 +2113,7 @@
       <c r="L43" s="25"/>
       <c r="M43" s="25"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -2110,7 +2127,7 @@
       <c r="L44" s="25"/>
       <c r="M44" s="25"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -2124,7 +2141,7 @@
       <c r="L45" s="25"/>
       <c r="M45" s="25"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="16"/>
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
@@ -2138,12 +2155,12 @@
       <c r="L46" s="28"/>
       <c r="M46" s="28"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="F48" s="23" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="49" spans="6:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="49" spans="6:12" ht="21" x14ac:dyDescent="0.25">
       <c r="F49" s="23" t="s">
         <v>105</v>
       </c>
@@ -2154,7 +2171,7 @@
       <c r="J49" s="49"/>
       <c r="K49" s="49"/>
     </row>
-    <row r="50" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F50" s="23" t="s">
         <v>92</v>
       </c>
@@ -2170,7 +2187,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F51" s="23" t="s">
         <v>106</v>
       </c>
@@ -2184,7 +2201,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="52" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F52" s="23" t="s">
         <v>107</v>
       </c>
@@ -2200,7 +2217,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="53" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F53" s="23"/>
       <c r="H53" s="7" t="s">
         <v>65</v>
@@ -2214,7 +2231,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="54" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F54" s="40"/>
       <c r="H54" s="9"/>
       <c r="I54" s="9"/>
@@ -2222,10 +2239,10 @@
       <c r="K54" s="15"/>
       <c r="L54" s="36"/>
     </row>
-    <row r="55" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F55" s="40"/>
     </row>
-    <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.25">
       <c r="H57" s="49" t="s">
         <v>66</v>
       </c>
@@ -2233,7 +2250,7 @@
       <c r="J57" s="49"/>
       <c r="K57" s="49"/>
     </row>
-    <row r="58" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H58" s="4" t="s">
         <v>58</v>
       </c>
@@ -2246,7 +2263,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H59" s="30"/>
       <c r="I59" s="30"/>
       <c r="J59" s="30"/>
@@ -2257,7 +2274,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="60" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H60" s="7" t="s">
         <v>67</v>
       </c>
@@ -2270,7 +2287,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="61" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H61" s="7" t="s">
         <v>68</v>
       </c>
@@ -2283,14 +2300,14 @@
         <v>220</v>
       </c>
     </row>
-    <row r="62" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H62" s="9"/>
       <c r="I62" s="9"/>
       <c r="J62" s="9"/>
       <c r="K62" s="15"/>
       <c r="L62" s="15"/>
     </row>
-    <row r="64" spans="6:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="64" spans="6:12" ht="19" x14ac:dyDescent="0.25">
       <c r="H64" s="50" t="s">
         <v>70</v>
       </c>
@@ -2299,7 +2316,7 @@
       <c r="K64" s="50"/>
       <c r="L64" s="50"/>
     </row>
-    <row r="65" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H65" s="32" t="s">
         <v>71</v>
       </c>
@@ -2310,7 +2327,7 @@
       </c>
       <c r="L65" s="52"/>
     </row>
-    <row r="66" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H66" s="14" t="s">
         <v>73</v>
       </c>
@@ -2321,7 +2338,7 @@
       </c>
       <c r="L66" s="8"/>
     </row>
-    <row r="67" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H67" s="14" t="s">
         <v>74</v>
       </c>
@@ -2332,14 +2349,14 @@
       </c>
       <c r="L67" s="8"/>
     </row>
-    <row r="68" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H68" s="14"/>
       <c r="I68" s="22"/>
       <c r="J68" s="22"/>
       <c r="K68" s="22"/>
       <c r="L68" s="8"/>
     </row>
-    <row r="69" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H69" s="15"/>
       <c r="I69" s="16"/>
       <c r="J69" s="16"/>
@@ -2368,12 +2385,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -2393,7 +2410,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2406,7 +2423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -2419,7 +2436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -2432,7 +2449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2453,12 +2470,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
@@ -2466,7 +2483,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -2474,7 +2491,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -2482,7 +2499,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -2490,7 +2507,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -2498,7 +2515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -2514,12 +2531,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>26</v>
       </c>
@@ -2530,7 +2547,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -2541,7 +2558,7 @@
         <v>37.799999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -2552,7 +2569,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -2563,7 +2580,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2574,7 +2591,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -2585,7 +2602,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2596,7 +2613,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>80</v>
       </c>
@@ -2609,25 +2626,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2690AB0E-8EB0-45FB-A556-DB8C8710C025}">
   <dimension ref="A1:M69"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
     <col min="2" max="2" width="7.33203125" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
     <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="8" max="8" width="14.5" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="7.6640625" customWidth="1"/>
-    <col min="11" max="11" width="37.88671875" customWidth="1"/>
-    <col min="12" max="12" width="14.44140625" customWidth="1"/>
-    <col min="13" max="13" width="13.44140625" customWidth="1"/>
+    <col min="11" max="11" width="66.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.5" customWidth="1"/>
+    <col min="13" max="13" width="13.5" customWidth="1"/>
     <col min="14" max="14" width="0.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
         <v>40</v>
       </c>
@@ -2643,7 +2660,7 @@
       <c r="J1" s="49"/>
       <c r="K1" s="49"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -2678,7 +2695,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -2691,7 +2708,7 @@
       <c r="K3" s="31"/>
       <c r="L3" s="34"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
@@ -2714,13 +2731,13 @@
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
       <c r="K4" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L4" s="35">
         <v>2500</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
@@ -2743,13 +2760,13 @@
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
       <c r="K5" s="14" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="L5" s="35">
         <v>450</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
@@ -2772,11 +2789,11 @@
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L6" s="35"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
@@ -2799,11 +2816,11 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="48" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L7" s="35"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
@@ -2820,9 +2837,15 @@
         <v>8250</v>
       </c>
       <c r="F8" s="12"/>
+      <c r="H8" s="58" t="s">
+        <v>121</v>
+      </c>
+      <c r="K8" s="59" t="s">
+        <v>122</v>
+      </c>
       <c r="L8" s="35"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
@@ -2839,13 +2862,17 @@
         <v>14500</v>
       </c>
       <c r="F9" s="12"/>
-      <c r="H9" s="7"/>
+      <c r="H9" s="7" t="s">
+        <v>123</v>
+      </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
-      <c r="K9" s="14"/>
+      <c r="K9" s="14" t="s">
+        <v>124</v>
+      </c>
       <c r="L9" s="35"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
@@ -2868,7 +2895,7 @@
       <c r="K10" s="14"/>
       <c r="L10" s="35"/>
     </row>
-    <row r="11" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -2893,7 +2920,7 @@
       </c>
       <c r="L11" s="35"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
@@ -2916,7 +2943,7 @@
       <c r="K12" s="14"/>
       <c r="L12" s="35"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -2929,7 +2956,7 @@
       <c r="K13" s="14"/>
       <c r="L13" s="35"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -2942,7 +2969,7 @@
       <c r="K14" s="14"/>
       <c r="L14" s="35"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="13"/>
@@ -2954,7 +2981,7 @@
       <c r="K15" s="15"/>
       <c r="L15" s="36"/>
     </row>
-    <row r="18" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="53" t="s">
         <v>41</v>
       </c>
@@ -2972,7 +2999,7 @@
       <c r="L18" s="55"/>
       <c r="M18" s="56"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
@@ -3010,7 +3037,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -3024,7 +3051,7 @@
       <c r="L20" s="21"/>
       <c r="M20" s="21"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>42</v>
       </c>
@@ -3062,7 +3089,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>43</v>
       </c>
@@ -3100,7 +3127,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>44</v>
       </c>
@@ -3138,7 +3165,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>45</v>
       </c>
@@ -3176,7 +3203,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>46</v>
       </c>
@@ -3192,7 +3219,9 @@
       <c r="E25" s="35">
         <v>26.58</v>
       </c>
-      <c r="F25" s="38"/>
+      <c r="F25" s="38">
+        <v>2600</v>
+      </c>
       <c r="H25" s="23" t="s">
         <v>46</v>
       </c>
@@ -3202,7 +3231,7 @@
       <c r="L25" s="25"/>
       <c r="M25" s="25"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>47</v>
       </c>
@@ -3218,7 +3247,9 @@
       <c r="E26" s="35">
         <v>26.34</v>
       </c>
-      <c r="F26" s="38"/>
+      <c r="F26" s="38">
+        <v>2600</v>
+      </c>
       <c r="H26" s="23" t="s">
         <v>47</v>
       </c>
@@ -3228,7 +3259,7 @@
       <c r="L26" s="25"/>
       <c r="M26" s="25"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>48</v>
       </c>
@@ -3244,7 +3275,9 @@
       <c r="E27" s="35">
         <v>26.34</v>
       </c>
-      <c r="F27" s="38"/>
+      <c r="F27" s="38">
+        <v>2600</v>
+      </c>
       <c r="H27" s="23" t="s">
         <v>48</v>
       </c>
@@ -3254,7 +3287,7 @@
       <c r="L27" s="25"/>
       <c r="M27" s="25"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>49</v>
       </c>
@@ -3270,7 +3303,9 @@
       <c r="E28" s="35">
         <v>25.01</v>
       </c>
-      <c r="F28" s="38"/>
+      <c r="F28" s="38">
+        <v>2600</v>
+      </c>
       <c r="H28" s="23" t="s">
         <v>49</v>
       </c>
@@ -3280,7 +3315,7 @@
       <c r="L28" s="25"/>
       <c r="M28" s="25"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>50</v>
       </c>
@@ -3296,7 +3331,9 @@
       <c r="E29" s="35">
         <v>35.57</v>
       </c>
-      <c r="F29" s="38"/>
+      <c r="F29" s="38">
+        <v>2600</v>
+      </c>
       <c r="H29" s="23" t="s">
         <v>50</v>
       </c>
@@ -3306,7 +3343,7 @@
       <c r="L29" s="25"/>
       <c r="M29" s="25"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>97</v>
       </c>
@@ -3322,7 +3359,9 @@
       <c r="E30" s="36">
         <v>40.56</v>
       </c>
-      <c r="F30" s="39"/>
+      <c r="F30" s="38">
+        <v>2600</v>
+      </c>
       <c r="H30" s="26"/>
       <c r="I30" s="26"/>
       <c r="J30" s="26"/>
@@ -3330,10 +3369,10 @@
       <c r="L30" s="28"/>
       <c r="M30" s="28"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="7"/>
     </row>
-    <row r="34" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" ht="19" x14ac:dyDescent="0.25">
       <c r="A34" s="53" t="s">
         <v>51</v>
       </c>
@@ -3351,7 +3390,7 @@
       <c r="L34" s="55"/>
       <c r="M34" s="56"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>0</v>
       </c>
@@ -3389,7 +3428,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -3403,7 +3442,7 @@
       <c r="L36" s="46"/>
       <c r="M36" s="21"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>42</v>
       </c>
@@ -3437,7 +3476,7 @@
       </c>
       <c r="M37" s="25"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>43</v>
       </c>
@@ -3471,7 +3510,7 @@
       </c>
       <c r="M38" s="25"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>44</v>
       </c>
@@ -3505,7 +3544,7 @@
       </c>
       <c r="M39" s="25"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>45</v>
       </c>
@@ -3539,7 +3578,7 @@
       </c>
       <c r="M40" s="25"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
         <v>46</v>
       </c>
@@ -3573,7 +3612,7 @@
       </c>
       <c r="M41" s="25"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
         <v>47</v>
       </c>
@@ -3597,7 +3636,7 @@
       <c r="L42" s="44"/>
       <c r="M42" s="25"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
@@ -3611,7 +3650,7 @@
       <c r="L43" s="25"/>
       <c r="M43" s="25"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -3625,7 +3664,7 @@
       <c r="L44" s="25"/>
       <c r="M44" s="25"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -3639,7 +3678,7 @@
       <c r="L45" s="25"/>
       <c r="M45" s="25"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="16"/>
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
@@ -3653,19 +3692,19 @@
       <c r="L46" s="28"/>
       <c r="M46" s="28"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="F48" s="23"/>
     </row>
-    <row r="49" spans="6:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="49" spans="6:12" ht="21" x14ac:dyDescent="0.25">
       <c r="F49" s="23"/>
-      <c r="H49" s="49" t="s">
-        <v>118</v>
-      </c>
-      <c r="I49" s="49"/>
-      <c r="J49" s="49"/>
-      <c r="K49" s="49"/>
-    </row>
-    <row r="50" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="H49" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="I49" s="57"/>
+      <c r="J49" s="57"/>
+      <c r="K49" s="57"/>
+    </row>
+    <row r="50" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F50" s="23"/>
       <c r="H50" s="4" t="s">
         <v>58</v>
@@ -3679,7 +3718,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F51" s="23"/>
       <c r="H51" s="30"/>
       <c r="I51" s="30"/>
@@ -3691,7 +3730,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F52" s="23"/>
       <c r="H52" s="7" t="s">
         <v>64</v>
@@ -3705,7 +3744,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="53" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F53" s="23"/>
       <c r="H53" s="7" t="s">
         <v>65</v>
@@ -3713,13 +3752,13 @@
       <c r="I53" s="7"/>
       <c r="J53" s="7"/>
       <c r="K53" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L53" s="35">
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F54" s="40"/>
       <c r="H54" s="9"/>
       <c r="I54" s="9"/>
@@ -3727,18 +3766,18 @@
       <c r="K54" s="15"/>
       <c r="L54" s="36"/>
     </row>
-    <row r="55" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F55" s="40"/>
     </row>
-    <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="H57" s="49" t="s">
+    <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.25">
+      <c r="H57" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="I57" s="49"/>
-      <c r="J57" s="49"/>
-      <c r="K57" s="49"/>
-    </row>
-    <row r="58" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="I57" s="57"/>
+      <c r="J57" s="57"/>
+      <c r="K57" s="57"/>
+    </row>
+    <row r="58" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H58" s="4" t="s">
         <v>58</v>
       </c>
@@ -3751,7 +3790,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H59" s="30"/>
       <c r="I59" s="30"/>
       <c r="J59" s="30"/>
@@ -3762,7 +3801,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="60" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H60" s="7" t="s">
         <v>67</v>
       </c>
@@ -3775,7 +3814,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="61" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H61" s="7" t="s">
         <v>68</v>
       </c>
@@ -3784,14 +3823,14 @@
       <c r="K61" s="14"/>
       <c r="L61" s="14"/>
     </row>
-    <row r="62" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H62" s="9"/>
       <c r="I62" s="9"/>
       <c r="J62" s="9"/>
       <c r="K62" s="15"/>
       <c r="L62" s="15"/>
     </row>
-    <row r="64" spans="6:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="64" spans="6:12" ht="19" x14ac:dyDescent="0.25">
       <c r="H64" s="50" t="s">
         <v>70</v>
       </c>
@@ -3800,7 +3839,7 @@
       <c r="K64" s="50"/>
       <c r="L64" s="50"/>
     </row>
-    <row r="65" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H65" s="32" t="s">
         <v>71</v>
       </c>
@@ -3811,18 +3850,18 @@
       </c>
       <c r="L65" s="52"/>
     </row>
-    <row r="66" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H66" s="14" t="s">
         <v>73</v>
       </c>
       <c r="I66" s="22"/>
       <c r="J66" s="22"/>
       <c r="K66" s="33" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L66" s="8"/>
     </row>
-    <row r="67" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H67" s="14" t="s">
         <v>74</v>
       </c>
@@ -3833,14 +3872,14 @@
       </c>
       <c r="L67" s="8"/>
     </row>
-    <row r="68" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H68" s="14"/>
       <c r="I68" s="22"/>
       <c r="J68" s="22"/>
       <c r="K68" s="22"/>
       <c r="L68" s="8"/>
     </row>
-    <row r="69" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="8:12" x14ac:dyDescent="0.2">
       <c r="H69" s="15"/>
       <c r="I69" s="16"/>
       <c r="J69" s="16"/>

</xml_diff>

<commit_message>
feat: update storage minimum fee to R650 and set mid-month discount window to 5th-24th
</commit_message>
<xml_diff>
--- a/WORKINGS FOR CURT APP PRICING.xlsx 20-05-2026.xlsx
+++ b/WORKINGS FOR CURT APP PRICING.xlsx 20-05-2026.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3AA3CF-2C82-DA4C-85C2-191D00D531EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-10020" windowWidth="38400" windowHeight="21600" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="National Costing" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -780,7 +780,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -795,6 +795,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -804,11 +807,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1138,12 +1136,12 @@
       <c r="D1" s="53"/>
       <c r="E1" s="53"/>
       <c r="F1" s="53"/>
-      <c r="H1" s="49" t="s">
+      <c r="H1" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -1481,14 +1479,14 @@
       <c r="D18" s="53"/>
       <c r="E18" s="53"/>
       <c r="F18" s="53"/>
-      <c r="H18" s="54" t="s">
+      <c r="H18" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="56"/>
+      <c r="I18" s="56"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="57"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
@@ -1844,14 +1842,14 @@
       <c r="D34" s="53"/>
       <c r="E34" s="53"/>
       <c r="F34" s="53"/>
-      <c r="H34" s="54" t="s">
+      <c r="H34" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55"/>
-      <c r="L34" s="55"/>
-      <c r="M34" s="56"/>
+      <c r="I34" s="56"/>
+      <c r="J34" s="56"/>
+      <c r="K34" s="56"/>
+      <c r="L34" s="56"/>
+      <c r="M34" s="57"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
@@ -2164,12 +2162,12 @@
       <c r="F49" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="H49" s="49" t="s">
+      <c r="H49" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="I49" s="49"/>
-      <c r="J49" s="49"/>
-      <c r="K49" s="49"/>
+      <c r="I49" s="54"/>
+      <c r="J49" s="54"/>
+      <c r="K49" s="54"/>
     </row>
     <row r="50" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F50" s="23" t="s">
@@ -2243,12 +2241,12 @@
       <c r="F55" s="40"/>
     </row>
     <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="H57" s="49" t="s">
+      <c r="H57" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="I57" s="49"/>
-      <c r="J57" s="49"/>
-      <c r="K57" s="49"/>
+      <c r="I57" s="54"/>
+      <c r="J57" s="54"/>
+      <c r="K57" s="54"/>
     </row>
     <row r="58" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H58" s="4" t="s">
@@ -2653,12 +2651,12 @@
       <c r="D1" s="53"/>
       <c r="E1" s="53"/>
       <c r="F1" s="53"/>
-      <c r="H1" s="49" t="s">
+      <c r="H1" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -2837,10 +2835,10 @@
         <v>8250</v>
       </c>
       <c r="F8" s="12"/>
-      <c r="H8" s="58" t="s">
+      <c r="H8" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="K8" s="59" t="s">
+      <c r="K8" s="14" t="s">
         <v>122</v>
       </c>
       <c r="L8" s="35"/>
@@ -2990,14 +2988,14 @@
       <c r="D18" s="53"/>
       <c r="E18" s="53"/>
       <c r="F18" s="53"/>
-      <c r="H18" s="54" t="s">
+      <c r="H18" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="56"/>
+      <c r="I18" s="56"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="57"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
@@ -3381,14 +3379,14 @@
       <c r="D34" s="53"/>
       <c r="E34" s="53"/>
       <c r="F34" s="53"/>
-      <c r="H34" s="54" t="s">
+      <c r="H34" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55"/>
-      <c r="L34" s="55"/>
-      <c r="M34" s="56"/>
+      <c r="I34" s="56"/>
+      <c r="J34" s="56"/>
+      <c r="K34" s="56"/>
+      <c r="L34" s="56"/>
+      <c r="M34" s="57"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
@@ -3697,12 +3695,12 @@
     </row>
     <row r="49" spans="6:12" ht="21" x14ac:dyDescent="0.25">
       <c r="F49" s="23"/>
-      <c r="H49" s="57" t="s">
+      <c r="H49" s="49" t="s">
         <v>117</v>
       </c>
-      <c r="I49" s="57"/>
-      <c r="J49" s="57"/>
-      <c r="K49" s="57"/>
+      <c r="I49" s="49"/>
+      <c r="J49" s="49"/>
+      <c r="K49" s="49"/>
     </row>
     <row r="50" spans="6:12" x14ac:dyDescent="0.2">
       <c r="F50" s="23"/>
@@ -3770,12 +3768,12 @@
       <c r="F55" s="40"/>
     </row>
     <row r="57" spans="6:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="H57" s="57" t="s">
+      <c r="H57" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="I57" s="57"/>
-      <c r="J57" s="57"/>
-      <c r="K57" s="57"/>
+      <c r="I57" s="49"/>
+      <c r="J57" s="49"/>
+      <c r="K57" s="49"/>
     </row>
     <row r="58" spans="6:12" x14ac:dyDescent="0.2">
       <c r="H58" s="4" t="s">

</xml_diff>